<commit_message>
Update Semana 10 materials: Enhance evaluation rubric, add new lab content, and restructure class resources
</commit_message>
<xml_diff>
--- a/Savio/datos_laboratorio.xlsx
+++ b/Savio/datos_laboratorio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecnoutb-my.sharepoint.com/personal/ksossa_utb_edu_co/Documents/cursos/Ciencias Básicas/Estadistica I/2.Material del curso/Datos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecnoutb-my.sharepoint.com/personal/ksossa_utb_edu_co/Documents/Github/estadistica-probabilidad-curso/Savio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{798C8F74-D59C-431B-90DD-5D59F884F623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BC4A463-652A-4B5D-BFE5-C3BB807E416E}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{798C8F74-D59C-431B-90DD-5D59F884F623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{220903AC-9BE0-4FAE-A600-A8444C5BAEF4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{656E9302-A581-40BC-9520-0ADD5111B459}"/>
   </bookViews>
@@ -48,12 +48,6 @@
   </si>
   <si>
     <t>ESTADÍSTICA I</t>
-  </si>
-  <si>
-    <t>A. Independientes</t>
-  </si>
-  <si>
-    <t>CORTE I DEFINITIVA (30%)</t>
   </si>
   <si>
     <t>EDAD</t>
@@ -149,13 +143,19 @@
     <t>ESTADISTICA II</t>
   </si>
   <si>
-    <t>EXAMEN1</t>
+    <t>CURSO</t>
   </si>
   <si>
-    <t>EXAMEN1 - puntos</t>
+    <t>Examen_1</t>
   </si>
   <si>
-    <t>CURSO</t>
+    <t>Examen_2</t>
+  </si>
+  <si>
+    <t>Definitiva</t>
+  </si>
+  <si>
+    <t>Puntos</t>
   </si>
 </sst>
 </file>
@@ -870,45 +870,45 @@
     <col min="12" max="12" width="19.81640625" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="39" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -938,16 +938,16 @@
         <v>176</v>
       </c>
       <c r="I2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="K2" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>15</v>
       </c>
       <c r="M2" s="10">
         <v>34</v>
@@ -980,16 +980,16 @@
         <v>167</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="M3" s="11">
         <v>43</v>
@@ -1022,16 +1022,16 @@
         <v>177</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M4" s="10">
         <v>33</v>
@@ -1064,16 +1064,16 @@
         <v>174</v>
       </c>
       <c r="I5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="K5" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L5" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M5" s="15">
         <v>15</v>
@@ -1106,16 +1106,16 @@
         <v>178</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M6" s="10">
         <v>23</v>
@@ -1148,16 +1148,16 @@
         <v>154</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M7" s="11">
         <v>35</v>
@@ -1190,16 +1190,16 @@
         <v>161</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="K8" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M8" s="10">
         <v>43</v>
@@ -1232,16 +1232,16 @@
         <v>153</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J9" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>15</v>
       </c>
       <c r="M9" s="11">
         <v>36</v>
@@ -1274,16 +1274,16 @@
         <v>168</v>
       </c>
       <c r="I10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K10" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="K10" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L10" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M10" s="10">
         <v>35</v>
@@ -1316,16 +1316,16 @@
         <v>172</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J11" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L11" s="11" t="s">
         <v>24</v>
-      </c>
-      <c r="K11" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L11" s="11" t="s">
-        <v>26</v>
       </c>
       <c r="M11" s="11">
         <v>32</v>
@@ -1358,16 +1358,16 @@
         <v>171</v>
       </c>
       <c r="I12" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="K12" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L12" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M12" s="10">
         <v>33</v>
@@ -1397,19 +1397,19 @@
         <v>70</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K13" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M13" s="15">
         <v>16</v>
@@ -1442,16 +1442,16 @@
         <v>174</v>
       </c>
       <c r="I14" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J14" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L14" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M14" s="10">
         <v>23</v>
@@ -1484,16 +1484,16 @@
         <v>162</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J15" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="M15" s="11">
         <v>21</v>
@@ -1526,16 +1526,16 @@
         <v>160</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J16" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="L16" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="M16" s="10">
         <v>29</v>
@@ -1568,16 +1568,16 @@
         <v>172</v>
       </c>
       <c r="I17" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J17" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L17" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M17" s="11">
         <v>41</v>
@@ -1610,16 +1610,16 @@
         <v>175</v>
       </c>
       <c r="I18" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K18" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L18" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M18" s="10">
         <v>30</v>
@@ -1652,16 +1652,16 @@
         <v>165</v>
       </c>
       <c r="I19" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J19" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K19" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M19" s="11">
         <v>41</v>
@@ -1694,16 +1694,16 @@
         <v>180</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J20" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M20" s="10">
         <v>33</v>
@@ -1736,16 +1736,16 @@
         <v>174</v>
       </c>
       <c r="I21" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K21" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J21" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="K21" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L21" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M21" s="11">
         <v>42</v>
@@ -1778,16 +1778,16 @@
         <v>182</v>
       </c>
       <c r="I22" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J22" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="K22" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L22" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M22" s="10">
         <v>38</v>
@@ -1820,16 +1820,16 @@
         <v>179</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J23" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="L23" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="K23" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="L23" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="M23" s="11">
         <v>25</v>
@@ -1862,16 +1862,16 @@
         <v>182</v>
       </c>
       <c r="I24" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J24" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K24" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J24" s="10" t="s">
+      <c r="L24" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="K24" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="L24" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="M24" s="10">
         <v>34</v>
@@ -1904,16 +1904,16 @@
         <v>174</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L25" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M25" s="11">
         <v>41</v>
@@ -1946,16 +1946,16 @@
         <v>177</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J26" s="10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K26" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L26" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M26" s="10">
         <v>41</v>
@@ -1988,16 +1988,16 @@
         <v>174</v>
       </c>
       <c r="I27" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K27" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J27" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="K27" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L27" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M27" s="11">
         <v>20</v>
@@ -2030,16 +2030,16 @@
         <v>165</v>
       </c>
       <c r="I28" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K28" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J28" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K28" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L28" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M28" s="10">
         <v>27</v>
@@ -2072,16 +2072,16 @@
         <v>177</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L29" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M29" s="15">
         <v>18</v>
@@ -2114,16 +2114,16 @@
         <v>167</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J30" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K30" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M30" s="10">
         <v>35</v>
@@ -2156,16 +2156,16 @@
         <v>165</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K31" s="11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M31" s="15">
         <v>50</v>
@@ -2198,16 +2198,16 @@
         <v>163</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J32" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L32" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="K32" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="L32" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="M32" s="10">
         <v>32</v>
@@ -2240,16 +2240,16 @@
         <v>160</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J33" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L33" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="K33" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="L33" s="11" t="s">
-        <v>15</v>
       </c>
       <c r="M33" s="11">
         <v>39</v>
@@ -2282,16 +2282,16 @@
         <v>163</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J34" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="K34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L34" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="K34" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="L34" s="10" t="s">
-        <v>15</v>
       </c>
       <c r="M34" s="10">
         <v>23</v>
@@ -2324,16 +2324,16 @@
         <v>168</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J35" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L35" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="K35" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="L35" s="11" t="s">
-        <v>15</v>
       </c>
       <c r="M35" s="11">
         <v>24</v>
@@ -2366,16 +2366,16 @@
         <v>174</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J36" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M36" s="10">
         <v>26</v>
@@ -2408,16 +2408,16 @@
         <v>168</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K37" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L37" s="11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M37" s="11">
         <v>29</v>
@@ -2450,16 +2450,16 @@
         <v>158</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J38" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K38" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L38" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M38" s="10">
         <v>25</v>
@@ -2492,16 +2492,16 @@
         <v>189</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K39" s="11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L39" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M39" s="11">
         <v>40</v>
@@ -2534,16 +2534,16 @@
         <v>178</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J40" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L40" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M40" s="10">
         <v>37</v>
@@ -2576,16 +2576,16 @@
         <v>155</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M41" s="11">
         <v>23</v>
@@ -2618,16 +2618,16 @@
         <v>178</v>
       </c>
       <c r="I42" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J42" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K42" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J42" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="K42" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L42" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M42" s="10">
         <v>37</v>
@@ -2660,16 +2660,16 @@
         <v>165</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J43" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="L43" s="11" t="s">
         <v>16</v>
-      </c>
-      <c r="K43" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L43" s="11" t="s">
-        <v>18</v>
       </c>
       <c r="M43" s="11">
         <v>37</v>
@@ -2702,16 +2702,16 @@
         <v>180</v>
       </c>
       <c r="I44" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J44" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K44" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J44" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K44" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L44" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M44" s="10">
         <v>38</v>
@@ -2744,16 +2744,16 @@
         <v>167</v>
       </c>
       <c r="I45" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J45" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K45" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J45" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="K45" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L45" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M45" s="11">
         <v>29</v>
@@ -2786,16 +2786,16 @@
         <v>175</v>
       </c>
       <c r="I46" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J46" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K46" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J46" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K46" s="10" t="s">
-        <v>14</v>
-      </c>
       <c r="L46" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M46" s="10">
         <v>28</v>
@@ -2828,16 +2828,16 @@
         <v>183</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K47" s="11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L47" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M47" s="11">
         <v>26</v>
@@ -2870,16 +2870,16 @@
         <v>164</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J48" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K48" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="L48" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="K48" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="L48" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="M48" s="10">
         <v>43</v>
@@ -2909,19 +2909,19 @@
         <v>65</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K49" s="11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L49" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M49" s="11">
         <v>27</v>
@@ -2954,16 +2954,16 @@
         <v>160</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J50" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L50" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M50" s="10">
         <v>39</v>
@@ -2996,16 +2996,16 @@
         <v>151</v>
       </c>
       <c r="I51" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J51" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J51" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K51" s="11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L51" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M51" s="15">
         <v>20</v>
@@ -3038,16 +3038,16 @@
         <v>164</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J52" s="10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M52" s="10">
         <v>35</v>
@@ -3080,16 +3080,16 @@
         <v>157</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K53" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L53" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M53" s="15">
         <v>20</v>
@@ -3122,16 +3122,16 @@
         <v>159</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J54" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K54" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L54" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M54" s="10">
         <v>31</v>
@@ -3164,16 +3164,16 @@
         <v>162</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K55" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L55" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M55" s="20">
         <v>47</v>
@@ -3203,19 +3203,19 @@
         <v>50</v>
       </c>
       <c r="H56" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K56" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L56" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M56" s="10">
         <v>27</v>
@@ -3248,16 +3248,16 @@
         <v>165</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K57" s="11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L57" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M57" s="11">
         <v>38</v>
@@ -3290,16 +3290,16 @@
         <v>157</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J58" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K58" s="10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L58" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M58" s="15">
         <v>12</v>
@@ -3332,16 +3332,16 @@
         <v>160</v>
       </c>
       <c r="I59" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J59" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J59" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K59" s="11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L59" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M59" s="11">
         <v>43</v>
@@ -3374,16 +3374,16 @@
         <v>163</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J60" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L60" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M60" s="10">
         <v>32</v>
@@ -3416,16 +3416,16 @@
         <v>159</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K61" s="11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L61" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M61" s="11">
         <v>43</v>
@@ -3436,7 +3436,7 @@
         <v>1629</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C62" s="6">
         <v>3.8870967741935485</v>
@@ -3457,16 +3457,16 @@
         <v>160</v>
       </c>
       <c r="I62" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J62" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J62" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="K62" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L62" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M62" s="15">
         <v>15</v>
@@ -3477,7 +3477,7 @@
         <v>1629</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C63" s="7">
         <v>4.5483870967741931</v>
@@ -3498,16 +3498,16 @@
         <v>160</v>
       </c>
       <c r="I63" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J63" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K63" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L63" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M63" s="11">
         <v>37</v>
@@ -3518,7 +3518,7 @@
         <v>1637</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C64" s="6">
         <v>3.9274193548387095</v>
@@ -3539,16 +3539,16 @@
         <v>170</v>
       </c>
       <c r="I64" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J64" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K64" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="J64" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K64" s="17" t="s">
-        <v>14</v>
-      </c>
       <c r="L64" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M64" s="10">
         <v>24</v>
@@ -3559,7 +3559,7 @@
         <v>1635</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C65" s="7">
         <v>3.32258064516129</v>
@@ -3580,16 +3580,16 @@
         <v>171</v>
       </c>
       <c r="I65" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="J65" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J65" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K65" s="19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L65" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M65" s="11">
         <v>27</v>
@@ -3600,7 +3600,7 @@
         <v>1634</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C66" s="6">
         <v>4.07258064516129</v>
@@ -3621,16 +3621,16 @@
         <v>168</v>
       </c>
       <c r="I66" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J66" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K66" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L66" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M66" s="10">
         <v>33</v>
@@ -3641,7 +3641,7 @@
         <v>1629</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C67" s="7">
         <v>3.943548387096774</v>
@@ -3662,16 +3662,16 @@
         <v>178</v>
       </c>
       <c r="I67" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="J67" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K67" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="J67" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="K67" s="19" t="s">
-        <v>14</v>
-      </c>
       <c r="L67" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M67" s="11">
         <v>50</v>
@@ -3682,7 +3682,7 @@
         <v>1636</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C68" s="6">
         <v>4.42741935483871</v>
@@ -3703,16 +3703,16 @@
         <v>167</v>
       </c>
       <c r="I68" s="17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K68" s="17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L68" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M68" s="10">
         <v>44</v>
@@ -3723,7 +3723,7 @@
         <v>1629</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C69" s="7">
         <v>4.42741935483871</v>
@@ -3744,16 +3744,16 @@
         <v>170</v>
       </c>
       <c r="I69" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="J69" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K69" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="J69" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="K69" s="19" t="s">
-        <v>14</v>
-      </c>
       <c r="L69" s="11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M69" s="11">
         <v>50</v>
@@ -3764,7 +3764,7 @@
         <v>1629</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C70" s="6">
         <v>4.75</v>
@@ -3785,16 +3785,16 @@
         <v>167</v>
       </c>
       <c r="I70" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J70" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K70" s="17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="L70" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M70" s="15">
         <v>20</v>
@@ -3805,7 +3805,7 @@
         <v>1629</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C71" s="7">
         <v>4.25</v>
@@ -3826,16 +3826,16 @@
         <v>165</v>
       </c>
       <c r="I71" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K71" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L71" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M71" s="11">
         <v>38</v>
@@ -3846,7 +3846,7 @@
         <v>1628</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C72" s="6">
         <v>4.024193548387097</v>
@@ -3867,16 +3867,16 @@
         <v>175</v>
       </c>
       <c r="I72" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J72" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J72" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="K72" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L72" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M72" s="10">
         <v>25</v>
@@ -3887,7 +3887,7 @@
         <v>1629</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C73" s="7">
         <v>4.508064516129032</v>
@@ -3908,16 +3908,16 @@
         <v>163</v>
       </c>
       <c r="I73" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J73" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K73" s="19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L73" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M73" s="11">
         <v>47</v>
@@ -3928,7 +3928,7 @@
         <v>1630</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C74" s="6">
         <v>4.669354838709677</v>
@@ -3949,16 +3949,16 @@
         <v>165</v>
       </c>
       <c r="I74" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J74" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J74" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="K74" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L74" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M74" s="10">
         <v>31</v>
@@ -3969,7 +3969,7 @@
         <v>1629</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C75" s="7">
         <v>4.57258064516129</v>
@@ -3990,16 +3990,16 @@
         <v>165</v>
       </c>
       <c r="I75" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K75" s="19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L75" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M75" s="11">
         <v>36</v>
@@ -4010,7 +4010,7 @@
         <v>1629</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C76" s="6">
         <v>4.193548387096774</v>
@@ -4031,16 +4031,16 @@
         <v>173</v>
       </c>
       <c r="I76" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J76" s="10">
         <v>0</v>
       </c>
       <c r="K76" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L76" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M76" s="10">
         <v>21</v>
@@ -4051,7 +4051,7 @@
         <v>1631</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C77" s="7">
         <v>4.346774193548387</v>
@@ -4072,16 +4072,16 @@
         <v>157</v>
       </c>
       <c r="I77" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K77" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L77" s="11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M77" s="11">
         <v>29</v>
@@ -4092,7 +4092,7 @@
         <v>1629</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C78" s="6">
         <v>3.32258064516129</v>
@@ -4113,16 +4113,16 @@
         <v>158</v>
       </c>
       <c r="I78" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J78" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K78" s="17" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L78" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M78" s="15">
         <v>15</v>
@@ -4133,7 +4133,7 @@
         <v>1629</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C79" s="7">
         <v>4.2661290322580641</v>
@@ -4154,16 +4154,16 @@
         <v>160</v>
       </c>
       <c r="I79" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K79" s="19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L79" s="11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M79" s="11">
         <v>50</v>
@@ -4174,7 +4174,7 @@
         <v>1629</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C80" s="6">
         <v>2.7419354838709675</v>
@@ -4195,16 +4195,16 @@
         <v>166</v>
       </c>
       <c r="I80" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J80" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J80" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="K80" s="17" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L80" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M80" s="15">
         <v>23</v>
@@ -4215,7 +4215,7 @@
         <v>1629</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C81" s="7">
         <v>4.57258064516129</v>
@@ -4236,16 +4236,16 @@
         <v>184</v>
       </c>
       <c r="I81" s="19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J81" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K81" s="19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L81" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M81" s="11">
         <v>50</v>
@@ -4256,7 +4256,7 @@
         <v>1629</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C82" s="6">
         <v>4.354838709677419</v>
@@ -4277,16 +4277,16 @@
         <v>160</v>
       </c>
       <c r="I82" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J82" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="K82" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L82" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="K82" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="L82" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="M82" s="10">
         <v>26</v>
@@ -4297,7 +4297,7 @@
         <v>1629</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C83" s="7">
         <v>4.088709677419355</v>
@@ -4318,16 +4318,16 @@
         <v>164</v>
       </c>
       <c r="I83" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K83" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L83" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M83" s="11">
         <v>36</v>
@@ -4338,7 +4338,7 @@
         <v>1629</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C84" s="6">
         <v>4.129032258064516</v>
@@ -4359,16 +4359,16 @@
         <v>173</v>
       </c>
       <c r="I84" s="17" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J84" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K84" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L84" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M84" s="10">
         <v>40</v>
@@ -4379,7 +4379,7 @@
         <v>1629</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C85" s="7">
         <v>4.2661290322580641</v>
@@ -4400,16 +4400,16 @@
         <v>163</v>
       </c>
       <c r="I85" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K85" s="19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L85" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M85" s="11">
         <v>42</v>
@@ -4420,7 +4420,7 @@
         <v>1629</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C86" s="6">
         <v>4.387096774193548</v>
@@ -4441,16 +4441,16 @@
         <v>171</v>
       </c>
       <c r="I86" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K86" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L86" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M86" s="10">
         <v>25</v>
@@ -4461,7 +4461,7 @@
         <v>1629</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C87" s="7">
         <v>4.064516129032258</v>
@@ -4482,16 +4482,16 @@
         <v>163</v>
       </c>
       <c r="I87" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="J87" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J87" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K87" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L87" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M87" s="11">
         <v>43</v>
@@ -4502,7 +4502,7 @@
         <v>1632</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C88" s="7">
         <v>4.3306451612903221</v>
@@ -4523,16 +4523,16 @@
         <v>155</v>
       </c>
       <c r="I88" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="J88" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="J88" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="K88" s="19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L88" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M88" s="11">
         <v>29</v>
@@ -4543,7 +4543,7 @@
         <v>1633</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C89" s="6">
         <v>4.508064516129032</v>
@@ -4564,16 +4564,16 @@
         <v>178</v>
       </c>
       <c r="I89" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="J89" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K89" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="J89" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="K89" s="17" t="s">
-        <v>14</v>
-      </c>
       <c r="L89" s="10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M89" s="15">
         <v>15</v>
@@ -4584,7 +4584,7 @@
         <v>1629</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C90" s="7">
         <v>4.411290322580645</v>
@@ -4605,16 +4605,16 @@
         <v>150</v>
       </c>
       <c r="I90" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K90" s="19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L90" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M90" s="11">
         <v>25</v>
@@ -4670,23 +4670,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="95cd6440-c325-41d3-9dea-77dcbf74ea34" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100E88377CD40F5B74B9CA2405AE39145E7" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ff64bb0892c17e9e9f3fd68b257a28c5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="95cd6440-c325-41d3-9dea-77dcbf74ea34" xmlns:ns4="2c610f96-7d7c-4f84-88ec-e1ea00be7fc1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7807e4ff0318acd8e1fad453fa84cb40" ns3:_="" ns4:_="">
     <xsd:import namespace="95cd6440-c325-41d3-9dea-77dcbf74ea34"/>
@@ -4939,10 +4922,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="95cd6440-c325-41d3-9dea-77dcbf74ea34" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DAF4711-0E9C-44C7-BF99-144233204335}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C1E6D00-ED5D-44FE-9684-4C48223B93B2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="95cd6440-c325-41d3-9dea-77dcbf74ea34"/>
+    <ds:schemaRef ds:uri="2c610f96-7d7c-4f84-88ec-e1ea00be7fc1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4965,20 +4976,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C1E6D00-ED5D-44FE-9684-4C48223B93B2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DAF4711-0E9C-44C7-BF99-144233204335}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="95cd6440-c325-41d3-9dea-77dcbf74ea34"/>
-    <ds:schemaRef ds:uri="2c610f96-7d7c-4f84-88ec-e1ea00be7fc1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>